<commit_message>
download pdf and json
and cleanup names
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>activity_identification</t>
+          <t>activity_title_objectives</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -762,19 +762,19 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Activity Identification</t>
+          <t>Activity Title and Learning Objectives</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>activity_for_review,activity_for_testing,approved_activity</t>
+          <t>all</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -794,35 +794,35 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>student_background</t>
+          <t>activity_description</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Student Background</t>
+          <t>Activity Description</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>activity_for_review,activity_for_testing,approved_activity</t>
+          <t>activity_idea</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>objectives_goals</t>
+          <t>student_background</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Learning Objectives &amp; Process Skill Goals</t>
+          <t>Student Background</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -888,26 +888,6 @@
       <c r="D11" s="5" t="inlineStr">
         <is>
           <t>activity_for_review,activity_for_testing,approved_activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>idea_details</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Activity Idea</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>activity_idea</t>
         </is>
       </c>
     </row>
@@ -922,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1017,43 +997,51 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>content_objectives_group</t>
+          <t>image_source_group</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>objectives_goals</t>
+          <t>image_source</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Learning Objective</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>+ Add learning objective</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
+          <t>+ Add image</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>approved_activity</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>image_authorship_mode == 'specify'</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>process_skills_group</t>
+          <t>content_objectives_group</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>objectives_goals</t>
+          <t>activity_title_objectives</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
@@ -1061,7 +1049,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Process Skill Goal</t>
+          <t>Content Objective</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -1070,7 +1058,7 @@
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>+ Add process skill goal</t>
+          <t>+ Add content objective</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr"/>
@@ -1079,103 +1067,33 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>image_source_group</t>
+          <t>process_skills_group</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>image_source</t>
+          <t>activity_title_objectives</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Process Objective</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>+ Add image</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>approved_activity</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>image_authorship_mode == 'specify'</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>idea_content_objectives_group</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>idea_details</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Content Objective</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>+ Add content objective</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>idea_process_skills_group</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>idea_details</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Process Objective</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
           <t>+ Add process objective</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1188,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1932,12 +1850,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>title_activity</t>
+          <t>activity_type</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>activity_identification</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr"/>
@@ -1946,15 +1864,19 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Title of Activity</t>
+          <t>Activity Type</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
+          <t>checkbox_group</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>learning_cycle:Learning Cycle|application:Application</t>
+        </is>
+      </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1984,12 +1906,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>activity_identification</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr"/>
       <c r="D15" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
@@ -2030,29 +1952,33 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>topic</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>activity_identification</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Topic</t>
+          <t>Setting</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
+          <t>checkbox_group</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>laboratory:Laboratory|classroom:Classroom</t>
+        </is>
+      </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2077,33 +2003,29 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>idea_activity_type</t>
+          <t>course</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Activity Type</t>
+          <t>Course (e.g., Physical Chemistry, General Biology)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>checkbox_group</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>learning_cycle:Learning Cycle|application:Application</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2128,31 +2050,31 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>idea_discipline</t>
+          <t>level</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
+          <t>classroom_context</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Discipline</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>select</t>
+          <t>checkbox_group</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>anatomy_physiology:Anatomy &amp; Physiology|astronomy:Astronomy|biology:Biology|chemistry:Chemistry|computer_science:Computer Science|economics:Economics|environmental_science:Environmental Science|exercise_science:Exercise Science|fine_arts:Fine Arts|general:General|general_education:General Education|general_science:General Science|language_arts:Language Arts|mathematics:Mathematics|music:Music|neuroscience:Neuroscience|physics:Physics|psychology:Psychology|statistics:Statistics</t>
+          <t>k5:K-5|middle:Middle School|high:High School|undergrad_intro:Undergraduate (introductory-level)|undergrad_upper:Undergraduate (upper-level)|grad:Graduate</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -2179,33 +2101,29 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>idea_setting</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
+          <t>activity_title_objectives</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr"/>
       <c r="D19" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>checkbox_group</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>laboratory:Laboratory|classroom:Classroom</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2230,21 +2148,25 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>course</t>
+          <t>objective_text</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr"/>
+          <t>activity_title_objectives</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>content_objectives_group</t>
+        </is>
+      </c>
       <c r="D20" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Course (e.g., Physical Chemistry, General Biology)</t>
+          <t>Content Objective</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -2260,7 +2182,7 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
@@ -2277,33 +2199,33 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>idea_level</t>
+          <t>skill_text</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>idea_context</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr"/>
+          <t>activity_title_objectives</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>process_skills_group</t>
+        </is>
+      </c>
       <c r="D21" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>Process Objective</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>checkbox_group</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>k5:K-5|middle:Middle School|high:High School|undergrad_intro:Undergraduate (introductory-level)|undergrad_upper:Undergraduate (upper-level)|grad:Graduate</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2311,7 +2233,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
@@ -2328,12 +2250,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>idea_title</t>
+          <t>idea_description</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>idea_details</t>
+          <t>activity_description</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr"/>
@@ -2342,12 +2264,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -2368,51 +2290,59 @@
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr"/>
-      <c r="M22" s="5" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>250 words or less</t>
+        </is>
+      </c>
       <c r="N22" s="5" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>idea_objective_text</t>
+          <t>image_authorship_mode</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>idea_details</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>idea_content_objectives_group</t>
-        </is>
-      </c>
+          <t>image_source</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr"/>
       <c r="D23" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Content Objective</t>
+          <t>Image Authorship</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>blanket_author:I am the author of all images in the activity|specify:Specify image authorship</t>
+        </is>
+      </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr"/>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>approved_activity</t>
+        </is>
+      </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
           <t>all</t>
@@ -2426,17 +2356,17 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>idea_skill_text</t>
+          <t>image_description</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>idea_details</t>
+          <t>image_source</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>idea_process_skills_group</t>
+          <t>image_source_group</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
@@ -2444,7 +2374,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Process Objective</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -2460,7 +2390,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
@@ -2470,36 +2400,48 @@
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr"/>
-      <c r="M24" s="5" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>A short description or filename identifying the image.</t>
+        </is>
+      </c>
       <c r="N24" s="5" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>idea_description</t>
+          <t>image_role</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>idea_details</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr"/>
+          <t>image_source</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>image_source_group</t>
+        </is>
+      </c>
       <c r="D25" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Image Credit</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>author:I am the author of this image|source:I am not the author of this image. Image source:</t>
+        </is>
+      </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2517,18 +2459,14 @@
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr"/>
-      <c r="M25" s="5" t="inlineStr">
-        <is>
-          <t>250 words or less</t>
-        </is>
-      </c>
+      <c r="M25" s="5" t="inlineStr"/>
       <c r="N25" s="5" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>image_authorship_mode</t>
+          <t>image_source_detail</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -2536,28 +2474,28 @@
           <t>image_source</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>image_source_group</t>
+        </is>
+      </c>
       <c r="D26" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Image Authorship</t>
+          <t>Source (URL or description)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>blanket_author:I am the author of all images in the activity|specify:Specify image authorship</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>IF_VISIBLE</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2565,17 +2503,17 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>approved_activity</t>
-        </is>
-      </c>
+      <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>image_role == 'source'</t>
+        </is>
+      </c>
       <c r="M26" s="5" t="inlineStr"/>
       <c r="N26" s="5" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr"/>
@@ -2583,36 +2521,32 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>image_description</t>
+          <t>ai_use_intro</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>image_source</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>image_source_group</t>
-        </is>
-      </c>
+          <t>ai_use</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
       <c r="D27" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Generative AI can support activity development, but it should support — not replace — your own instructional design, disciplinary judgment, and critical thinking. As AI plays a larger role in producing content, the expectation for your review, verification, and disclosure increases. Select the level that best describes how AI was used in developing this activity. Routine or Supportive use covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed. Substantive Developmental use means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification. Extensive Generative use means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>info</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2627,36 +2561,28 @@
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr"/>
-      <c r="M27" s="5" t="inlineStr">
-        <is>
-          <t>A short description or filename identifying the image.</t>
-        </is>
-      </c>
+      <c r="M27" s="5" t="inlineStr"/>
       <c r="N27" s="5" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>image_role</t>
+          <t>ai_use_level</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>image_source</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>image_source_group</t>
-        </is>
-      </c>
+          <t>ai_use</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr"/>
       <c r="D28" s="5" t="n">
         <v>2</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Image Credit</t>
+          <t>Level of AI use</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2666,7 +2592,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>author:I am the author of this image|source:I am not the author of this image. Image source:</t>
+          <t>no_ai:No AI was used|routine:Routine or Supportive use|substantive:Substantive development use|extensive:Extensive generative AI use</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2693,36 +2619,32 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>image_source_detail</t>
+          <t>ai_responsibility_statement</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>image_source</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>image_source_group</t>
-        </is>
-      </c>
+          <t>ai_use</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
       <c r="D29" s="5" t="n">
         <v>3</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Source (URL or description)</t>
+          <t>Author Responsibility Statement: By selecting this level, I affirm that I have critically reviewed, verified, and substantively revised any AI-assisted content in this activity. My own intellectual and creative contribution to this activity is substantial enough that I hold copyright in the final work, and I accept full responsibility for the accuracy, originality, instructional design, and POGIL alignment of the submitted activity.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>info</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>IF_VISIBLE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2738,7 +2660,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>image_role == 'source'</t>
+          <t>ai_use_level in [substantive,extensive]</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr"/>
@@ -2748,7 +2670,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>ai_use_intro</t>
+          <t>ai_responsibility_checkbox</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -2758,22 +2680,26 @@
       </c>
       <c r="C30" s="5" t="inlineStr"/>
       <c r="D30" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Generative AI can support activity development, but it should support — not replace — your own instructional design, disciplinary judgment, and critical thinking. As AI plays a larger role in producing content, the expectation for your review, verification, and disclosure increases. Select the level that best describes how AI was used in developing this activity. Routine or Supportive use covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed. Substantive Developmental use means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification. Extensive Generative use means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
+          <t>Affirmation</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>info</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr"/>
+          <t>checkbox_group</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>affirmed:I affirm the statement above.</t>
+        </is>
+      </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>IF_VISIBLE</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -2787,7 +2713,11 @@
           <t>all</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>ai_use_level in [substantive,extensive]</t>
+        </is>
+      </c>
       <c r="M30" s="5" t="inlineStr"/>
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
@@ -2795,7 +2725,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>ai_use_level</t>
+          <t>ai_use_description</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -2805,26 +2735,22 @@
       </c>
       <c r="C31" s="5" t="inlineStr"/>
       <c r="D31" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Level of AI use</t>
+          <t>Briefly describe how AI was used in developing this activity.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>no_ai:No AI was used|routine:Routine or Supportive use|substantive:Substantive development use|extensive:Extensive generative AI use</t>
-        </is>
-      </c>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>IF_VISIBLE</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2838,7 +2764,11 @@
           <t>all</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>ai_use_level in [substantive,extensive]</t>
+        </is>
+      </c>
       <c r="M31" s="5" t="inlineStr"/>
       <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr"/>
@@ -2846,32 +2776,36 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>ai_responsibility_statement</t>
+          <t>q2</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>ai_use</t>
+          <t>student_background</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr"/>
       <c r="D32" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Author Responsibility Statement: By selecting this level, I affirm that I have critically reviewed, verified, and substantively revised any AI-assisted content in this activity. My own intellectual and creative contribution to this activity is substantial enough that I hold copyright in the final work, and I accept full responsibility for the accuracy, originality, instructional design, and POGIL alignment of the submitted activity.</t>
+          <t>Have students used and/or reviewed this activity?</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>info</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr"/>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>yes:Yes|no:No</t>
+        </is>
+      </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -2885,11 +2819,7 @@
           <t>all</t>
         </is>
       </c>
-      <c r="L32" s="5" t="inlineStr">
-        <is>
-          <t>ai_use_level in [substantive,extensive]</t>
-        </is>
-      </c>
+      <c r="L32" s="5" t="inlineStr"/>
       <c r="M32" s="5" t="inlineStr"/>
       <c r="N32" s="5" t="inlineStr"/>
       <c r="O32" s="5" t="inlineStr"/>
@@ -2897,36 +2827,32 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>ai_responsibility_checkbox</t>
+          <t>q3a</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>ai_use</t>
+          <t>student_background</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr"/>
       <c r="D33" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Affirmation</t>
+          <t>Key knowledge students should have as a prerequisite.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>checkbox_group</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>affirmed:I affirm the statement above.</t>
-        </is>
-      </c>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>IF_VISIBLE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -2940,11 +2866,7 @@
           <t>all</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>ai_use_level in [substantive,extensive]</t>
-        </is>
-      </c>
+      <c r="L33" s="5" t="inlineStr"/>
       <c r="M33" s="5" t="inlineStr"/>
       <c r="N33" s="5" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr"/>
@@ -2952,21 +2874,21 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>ai_use_description</t>
+          <t>q3b</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>ai_use</t>
+          <t>student_background</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr"/>
       <c r="D34" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Briefly describe how AI was used in developing this activity.</t>
+          <t>Knowledge students are not expected to have prior to activity.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2977,7 +2899,7 @@
       <c r="G34" s="5" t="inlineStr"/>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>IF_VISIBLE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2991,11 +2913,7 @@
           <t>all</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>ai_use_level in [substantive,extensive]</t>
-        </is>
-      </c>
+      <c r="L34" s="5" t="inlineStr"/>
       <c r="M34" s="5" t="inlineStr"/>
       <c r="N34" s="5" t="inlineStr"/>
       <c r="O34" s="5" t="inlineStr"/>
@@ -3003,12 +2921,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>q2</t>
+          <t>approval_testing_evidence</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>student_background</t>
+          <t>approval_evidence</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr"/>
@@ -3017,19 +2935,15 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Have students used and/or reviewed this activity?</t>
+          <t>Provide evidence that this activity has been tested in the classroom, and describe how it has been revised based on that feedback.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>radio</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>yes:Yes|no:No</t>
-        </is>
-      </c>
+          <t>textarea</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr"/>
       <c r="H35" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -3047,154 +2961,13 @@
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr"/>
-      <c r="M35" s="5" t="inlineStr"/>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Include student performance data, instructor observations, or facilitator notes as applicable.</t>
+        </is>
+      </c>
       <c r="N35" s="5" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>q3a</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>student_background</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr"/>
-      <c r="D36" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Key knowledge students should have as a prerequisite.</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr"/>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J36" s="5" t="inlineStr"/>
-      <c r="K36" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="L36" s="5" t="inlineStr"/>
-      <c r="M36" s="5" t="inlineStr"/>
-      <c r="N36" s="5" t="inlineStr"/>
-      <c r="O36" s="5" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>q3b</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>student_background</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Knowledge students are not expected to have prior to activity.</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr"/>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="L37" s="5" t="inlineStr"/>
-      <c r="M37" s="5" t="inlineStr"/>
-      <c r="N37" s="5" t="inlineStr"/>
-      <c r="O37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>approval_testing_evidence</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>approval_evidence</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr"/>
-      <c r="D38" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Provide evidence that this activity has been tested in the classroom, and describe how it has been revised based on that feedback.</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>textarea</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J38" s="5" t="inlineStr"/>
-      <c r="K38" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="L38" s="5" t="inlineStr"/>
-      <c r="M38" s="5" t="inlineStr">
-        <is>
-          <t>Include student performance data, instructor observations, or facilitator notes as applicable.</t>
-        </is>
-      </c>
-      <c r="N38" s="5" t="inlineStr"/>
-      <c r="O38" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: pdf page breaks
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA63C45-9A0F-594A-973D-7D2A2E952DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CEB753-241D-9645-88F7-E62834C8650D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="189">
   <si>
     <t>PAC Activity Submission Form — Structure Specification</t>
   </si>
@@ -598,6 +598,9 @@
 • &lt;b&gt;Routine or Supportive use&lt;/b&gt; covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed.
 • &lt;b&gt;Substantive Developmental use&lt;/b&gt; means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification.
 • &lt;b&gt;Extensive Generative use&lt;/b&gt; means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
+  </si>
+  <si>
+    <t>Activity type and classroom context on new page</t>
   </si>
 </sst>
 </file>
@@ -2715,7 +2718,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2750,6 +2753,17 @@
         <v>184</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>188</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add info box
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CEB753-241D-9645-88F7-E62834C8650D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B4038F-0DC0-C542-9BBC-8F85817160D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="191">
   <si>
     <t>PAC Activity Submission Form — Structure Specification</t>
   </si>
@@ -339,36 +339,24 @@
     <t>activity_document</t>
   </si>
   <si>
-    <t>Activity</t>
-  </si>
-  <si>
     <t>yes:Activity</t>
   </si>
   <si>
     <t>toc_graphic</t>
   </si>
   <si>
-    <t>TOC Graphic</t>
-  </si>
-  <si>
     <t>yes:TOC Graphic</t>
   </si>
   <si>
     <t>answer_key</t>
   </si>
   <si>
-    <t>Student Answers (Key)</t>
-  </si>
-  <si>
     <t>yes:Student Answers (Key)</t>
   </si>
   <si>
     <t>facilitation_guide</t>
   </si>
   <si>
-    <t>Facilitation Guide</t>
-  </si>
-  <si>
     <t>yes:Facilitation Guide</t>
   </si>
   <si>
@@ -594,13 +582,31 @@
     <t>check_list</t>
   </si>
   <si>
+    <t>Activity type and classroom context on new page</t>
+  </si>
+  <si>
     <t>Generative AI can support activity development, but it should support — not replace — your own instructional design, disciplinary judgment, and critical thinking. As AI plays a larger role in producing content, the expectation for your review, verification, and disclosure increases. Select the level that best describes how AI was used in developing this activity.
-• &lt;b&gt;Routine or Supportive use&lt;/b&gt; covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed.
-• &lt;b&gt;Substantive Developmental use&lt;/b&gt; means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification.
-• &lt;b&gt;Extensive Generative use&lt;/b&gt; means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
-  </si>
-  <si>
-    <t>Activity type and classroom context on new page</t>
+• ROUTINE or SUPPORTIVE use covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed.
+• SUBSTANTIVE DEVELOPMENTAL use means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification.
+• EXTENSIVE GENERATIVE use means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
+  </si>
+  <si>
+    <t>check_list_intro</t>
+  </si>
+  <si>
+    <t>Activity (PDF)</t>
+  </si>
+  <si>
+    <t>TOC Graphic (PNG)</t>
+  </si>
+  <si>
+    <t>Student Answers / Key (PDF)</t>
+  </si>
+  <si>
+    <t>Facilitation Guide (PDF)</t>
+  </si>
+  <si>
+    <t>The following documents will be required during the upload. Requred documents are marked *. Ensure you have each required document in the indicated file format. (The submission form pdf and json are created by this web app when you click download.)</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1180,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B4" s="5">
         <v>12</v>
@@ -1436,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1616,28 +1622,26 @@
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="70" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>95</v>
+        <v>185</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5">
         <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>96</v>
+        <v>190</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>97</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="G5" s="5"/>
       <c r="H5" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>85</v>
@@ -1653,23 +1657,23 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5">
         <v>2</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>84</v>
@@ -1686,35 +1690,33 @@
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5">
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="J7" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
         <v>32</v>
       </c>
@@ -1725,23 +1727,23 @@
     </row>
     <row r="8" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5">
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>85</v>
@@ -1762,23 +1764,23 @@
     </row>
     <row r="9" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5">
         <v>5</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>108</v>
+        <v>187</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>85</v>
@@ -1797,25 +1799,25 @@
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
     </row>
-    <row r="10" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5">
         <v>6</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>111</v>
+        <v>188</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>85</v>
@@ -1824,7 +1826,7 @@
         <v>85</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>113</v>
+        <v>45</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>32</v>
@@ -1834,33 +1836,35 @@
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>60</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="C11" s="5"/>
       <c r="D11" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>115</v>
+        <v>189</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G11" s="5"/>
+        <v>92</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>108</v>
+      </c>
       <c r="H11" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="J11" s="5"/>
+        <v>85</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>109</v>
+      </c>
       <c r="K11" s="5" t="s">
         <v>32</v>
       </c>
@@ -1871,7 +1875,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>30</v>
@@ -1880,13 +1884,13 @@
         <v>60</v>
       </c>
       <c r="D12" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5" t="s">
@@ -1906,7 +1910,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>30</v>
@@ -1915,20 +1919,20 @@
         <v>60</v>
       </c>
       <c r="D13" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
@@ -1939,28 +1943,28 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
     </row>
-    <row r="14" spans="1:15" ht="70" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="D14" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>125</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="G14" s="5"/>
       <c r="H14" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>85</v>
@@ -1970,31 +1974,29 @@
         <v>32</v>
       </c>
       <c r="L14" s="5"/>
-      <c r="M14" s="5" t="s">
-        <v>185</v>
-      </c>
+      <c r="M14" s="5"/>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
     </row>
-    <row r="15" spans="1:15" ht="140" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" ht="70" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>128</v>
+        <v>92</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>84</v>
@@ -2007,29 +2009,31 @@
         <v>32</v>
       </c>
       <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="M15" s="5" t="s">
+        <v>181</v>
+      </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" ht="140" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>84</v>
@@ -2048,22 +2052,24 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G17" s="5"/>
+        <v>92</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>128</v>
+      </c>
       <c r="H17" s="5" t="s">
         <v>84</v>
       </c>
@@ -2079,26 +2085,24 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>137</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="G18" s="5"/>
       <c r="H18" s="5" t="s">
         <v>84</v>
       </c>
@@ -2114,24 +2118,26 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>28</v>
+        <v>131</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G19" s="5"/>
+        <v>92</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>84</v>
       </c>
@@ -2149,29 +2155,27 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>139</v>
+        <v>28</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>67</v>
-      </c>
+      <c r="C20" s="5"/>
       <c r="D20" s="5">
         <v>1</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>68</v>
+        <v>134</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="5" t="s">
         <v>84</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5" t="s">
@@ -2184,22 +2188,22 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D21" s="5">
         <v>1</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
@@ -2219,116 +2223,114 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="5"/>
+        <v>36</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="D22" s="5">
         <v>1</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="5" t="s">
         <v>84</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L22" s="5"/>
-      <c r="M22" s="5" t="s">
-        <v>144</v>
-      </c>
+      <c r="M22" s="5"/>
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5">
         <v>1</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>147</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="J23" s="5" t="s">
-        <v>48</v>
-      </c>
+      <c r="J23" s="5"/>
       <c r="K23" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
+      <c r="M23" s="5" t="s">
+        <v>140</v>
+      </c>
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="C24" s="5"/>
       <c r="D24" s="5">
         <v>1</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>64</v>
+        <v>142</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G24" s="5"/>
+        <v>82</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>143</v>
+      </c>
       <c r="H24" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="J24" s="5"/>
+      <c r="J24" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="K24" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L24" s="5"/>
-      <c r="M24" s="5" t="s">
-        <v>149</v>
-      </c>
+      <c r="M24" s="5"/>
       <c r="N24" s="5"/>
       <c r="O24" s="5"/>
     </row>
     <row r="25" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>49</v>
@@ -2337,17 +2339,15 @@
         <v>63</v>
       </c>
       <c r="D25" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>152</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
         <v>84</v>
       </c>
@@ -2359,13 +2359,15 @@
         <v>32</v>
       </c>
       <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
+      <c r="M25" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
     </row>
     <row r="26" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>49</v>
@@ -2374,17 +2376,19 @@
         <v>63</v>
       </c>
       <c r="D26" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G26" s="5"/>
+        <v>82</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>148</v>
+      </c>
       <c r="H26" s="5" t="s">
-        <v>155</v>
+        <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>85</v>
@@ -2393,33 +2397,33 @@
       <c r="K26" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L26" s="5" t="s">
-        <v>156</v>
-      </c>
+      <c r="L26" s="5"/>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="1:15" ht="238" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="5"/>
+        <v>49</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="D27" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>187</v>
+        <v>150</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>85</v>
+        <v>151</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>85</v>
@@ -2428,33 +2432,33 @@
       <c r="K27" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L27" s="5"/>
+      <c r="L27" s="5" t="s">
+        <v>152</v>
+      </c>
       <c r="M27" s="5"/>
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ht="238" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>161</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>85</v>
@@ -2468,26 +2472,28 @@
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
     </row>
-    <row r="29" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G29" s="5"/>
+        <v>82</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="H29" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>85</v>
@@ -2496,35 +2502,31 @@
       <c r="K29" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L29" s="5" t="s">
-        <v>164</v>
-      </c>
+      <c r="L29" s="5"/>
       <c r="M29" s="5"/>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
     </row>
-    <row r="30" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ht="112" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>167</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="G30" s="5"/>
       <c r="H30" s="5" t="s">
-        <v>155</v>
+        <v>85</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>85</v>
@@ -2534,7 +2536,7 @@
         <v>32</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
@@ -2542,24 +2544,26 @@
     </row>
     <row r="31" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G31" s="5"/>
+        <v>92</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>163</v>
+      </c>
       <c r="H31" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>85</v>
@@ -2569,34 +2573,32 @@
         <v>32</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
       <c r="O31" s="5"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>172</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="G32" s="5"/>
       <c r="H32" s="5" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>85</v>
@@ -2605,29 +2607,33 @@
       <c r="K32" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L32" s="5"/>
+      <c r="L32" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G33" s="5"/>
+        <v>82</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>168</v>
+      </c>
       <c r="H33" s="5" t="s">
         <v>84</v>
       </c>
@@ -2643,22 +2649,22 @@
       <c r="N33" s="5"/>
       <c r="O33" s="5"/>
     </row>
-    <row r="34" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
@@ -2676,22 +2682,22 @@
       <c r="N34" s="5"/>
       <c r="O34" s="5"/>
     </row>
-    <row r="35" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
@@ -2705,11 +2711,44 @@
         <v>32</v>
       </c>
       <c r="L35" s="5"/>
-      <c r="M35" s="5" t="s">
-        <v>179</v>
-      </c>
+      <c r="M35" s="5"/>
       <c r="N35" s="5"/>
       <c r="O35" s="5"/>
+    </row>
+    <row r="36" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5">
+        <v>1</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2729,16 +2768,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -2750,18 +2789,18 @@
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: AI text formatting
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B4038F-0DC0-C542-9BBC-8F85817160D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AB113F-21B3-DF47-903B-CEE796055818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -339,27 +339,15 @@
     <t>activity_document</t>
   </si>
   <si>
-    <t>yes:Activity</t>
-  </si>
-  <si>
     <t>toc_graphic</t>
   </si>
   <si>
-    <t>yes:TOC Graphic</t>
-  </si>
-  <si>
     <t>answer_key</t>
   </si>
   <si>
-    <t>yes:Student Answers (Key)</t>
-  </si>
-  <si>
     <t>facilitation_guide</t>
   </si>
   <si>
-    <t>yes:Facilitation Guide</t>
-  </si>
-  <si>
     <t>activity_for_testing,approved_activity</t>
   </si>
   <si>
@@ -462,9 +450,6 @@
     <t>Image Authorship</t>
   </si>
   <si>
-    <t>blanket_author:I am the author of all images in the activity|specify:Specify image authorship</t>
-  </si>
-  <si>
     <t>image_description</t>
   </si>
   <si>
@@ -585,28 +570,44 @@
     <t>Activity type and classroom context on new page</t>
   </si>
   <si>
-    <t>Generative AI can support activity development, but it should support — not replace — your own instructional design, disciplinary judgment, and critical thinking. As AI plays a larger role in producing content, the expectation for your review, verification, and disclosure increases. Select the level that best describes how AI was used in developing this activity.
+    <t>check_list_intro</t>
+  </si>
+  <si>
+    <t>Activity (PDF)</t>
+  </si>
+  <si>
+    <t>TOC Graphic (PNG)</t>
+  </si>
+  <si>
+    <t>Student Answers / Key (PDF)</t>
+  </si>
+  <si>
+    <t>Facilitation Guide (PDF)</t>
+  </si>
+  <si>
+    <t>The following documents will be required during the upload. Requred documents are marked *. Ensure you have each required document in the indicated file format. (The submission form pdf and json are created by this web app when you click download.)</t>
+  </si>
+  <si>
+    <t>yes:Activity (PDF)</t>
+  </si>
+  <si>
+    <t>yes:TOC Graphic (PNG)</t>
+  </si>
+  <si>
+    <t>yes:Student Answers / Key (PDF)</t>
+  </si>
+  <si>
+    <t>yes:Facilitation Guide (PDF)</t>
+  </si>
+  <si>
+    <t>blanket_author:I am the author of all images in the activity|specify:Specify image authorship individually</t>
+  </si>
+  <si>
+    <t>Generative AI can support activity development, but it should support — not replace — your own instructional design, disciplinary judgment, and critical thinking. As AI plays a larger role in producing content, the expectation for your review, verification, and disclosure increases. Three levels of AI use are
 • ROUTINE or SUPPORTIVE use covers things like brainstorming, wording suggestions, grammar/clarity checks, or formatting on work you conceived and directed.
 • SUBSTANTIVE DEVELOPMENTAL use means AI helped develop or revise real components — drafting objectives, generating questions from your objectives, building datasets, or suggesting scaffolding — requiring your careful review and verification.
-• EXTENSIVE GENERATIVE use means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.</t>
-  </si>
-  <si>
-    <t>check_list_intro</t>
-  </si>
-  <si>
-    <t>Activity (PDF)</t>
-  </si>
-  <si>
-    <t>TOC Graphic (PNG)</t>
-  </si>
-  <si>
-    <t>Student Answers / Key (PDF)</t>
-  </si>
-  <si>
-    <t>Facilitation Guide (PDF)</t>
-  </si>
-  <si>
-    <t>The following documents will be required during the upload. Requred documents are marked *. Ensure you have each required document in the indicated file format. (The submission form pdf and json are created by this web app when you click download.)</t>
+• EXTENSIVE GENERATIVE use means AI generated substantial portions of the activity (e.g. a full question sequence or draft) with limited initial input from you.
+ Select the level that best describes how AI was used in developing this activity.</t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1181,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B4" s="5">
         <v>12</v>
@@ -1624,20 +1625,20 @@
     </row>
     <row r="5" spans="1:15" ht="70" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5">
         <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5" t="s">
@@ -1660,7 +1661,7 @@
         <v>95</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5">
@@ -1695,7 +1696,7 @@
         <v>98</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5">
@@ -1730,20 +1731,20 @@
         <v>101</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5">
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>102</v>
+        <v>185</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>85</v>
@@ -1764,23 +1765,23 @@
     </row>
     <row r="9" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5">
         <v>5</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>104</v>
+        <v>186</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>85</v>
@@ -1801,23 +1802,23 @@
     </row>
     <row r="10" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5">
         <v>6</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>106</v>
+        <v>187</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>85</v>
@@ -1838,23 +1839,23 @@
     </row>
     <row r="11" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5">
         <v>7</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>108</v>
+        <v>188</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>85</v>
@@ -1863,7 +1864,7 @@
         <v>85</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>32</v>
@@ -1875,7 +1876,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>30</v>
@@ -1887,10 +1888,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5" t="s">
@@ -1910,7 +1911,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>30</v>
@@ -1922,10 +1923,10 @@
         <v>2</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5" t="s">
@@ -1945,7 +1946,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>30</v>
@@ -1957,10 +1958,10 @@
         <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5" t="s">
@@ -1980,7 +1981,7 @@
     </row>
     <row r="15" spans="1:15" ht="70" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>38</v>
@@ -1990,13 +1991,13 @@
         <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>84</v>
@@ -2010,14 +2011,14 @@
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="5" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
     </row>
     <row r="16" spans="1:15" ht="140" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>38</v>
@@ -2027,13 +2028,13 @@
         <v>3</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>84</v>
@@ -2052,7 +2053,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>38</v>
@@ -2062,13 +2063,13 @@
         <v>4</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>84</v>
@@ -2087,7 +2088,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>38</v>
@@ -2097,10 +2098,10 @@
         <v>5</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5" t="s">
@@ -2120,7 +2121,7 @@
     </row>
     <row r="19" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>38</v>
@@ -2130,13 +2131,13 @@
         <v>6</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>84</v>
@@ -2165,10 +2166,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="5" t="s">
@@ -2188,7 +2189,7 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>36</v>
@@ -2203,7 +2204,7 @@
         <v>68</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
@@ -2223,7 +2224,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>36</v>
@@ -2238,7 +2239,7 @@
         <v>71</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="5" t="s">
@@ -2258,7 +2259,7 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>40</v>
@@ -2268,10 +2269,10 @@
         <v>1</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
@@ -2286,14 +2287,14 @@
       </c>
       <c r="L23" s="5"/>
       <c r="M23" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>49</v>
@@ -2303,13 +2304,13 @@
         <v>1</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>82</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>143</v>
+        <v>189</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>85</v>
@@ -2330,7 +2331,7 @@
     </row>
     <row r="25" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>49</v>
@@ -2345,7 +2346,7 @@
         <v>64</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
@@ -2360,14 +2361,14 @@
       </c>
       <c r="L25" s="5"/>
       <c r="M25" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
     </row>
     <row r="26" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>49</v>
@@ -2379,13 +2380,13 @@
         <v>2</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>82</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>84</v>
@@ -2404,7 +2405,7 @@
     </row>
     <row r="27" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>49</v>
@@ -2416,14 +2417,14 @@
         <v>3</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>85</v>
@@ -2433,15 +2434,15 @@
         <v>32</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="M27" s="5"/>
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="1:15" ht="238" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ht="319" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>51</v>
@@ -2451,10 +2452,10 @@
         <v>1</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
@@ -2474,7 +2475,7 @@
     </row>
     <row r="29" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>51</v>
@@ -2484,13 +2485,13 @@
         <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>82</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>84</v>
@@ -2509,7 +2510,7 @@
     </row>
     <row r="30" spans="1:15" ht="112" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>51</v>
@@ -2519,10 +2520,10 @@
         <v>3</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="5" t="s">
@@ -2536,7 +2537,7 @@
         <v>32</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
@@ -2544,7 +2545,7 @@
     </row>
     <row r="31" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>51</v>
@@ -2554,16 +2555,16 @@
         <v>4</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>92</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>85</v>
@@ -2573,7 +2574,7 @@
         <v>32</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -2581,7 +2582,7 @@
     </row>
     <row r="32" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>51</v>
@@ -2591,14 +2592,14 @@
         <v>5</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>85</v>
@@ -2608,7 +2609,7 @@
         <v>32</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -2616,7 +2617,7 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>43</v>
@@ -2626,13 +2627,13 @@
         <v>1</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>82</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="H33" s="5" t="s">
         <v>84</v>
@@ -2651,7 +2652,7 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>43</v>
@@ -2661,10 +2662,10 @@
         <v>2</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
@@ -2684,7 +2685,7 @@
     </row>
     <row r="35" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>43</v>
@@ -2694,10 +2695,10 @@
         <v>3</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
@@ -2717,7 +2718,7 @@
     </row>
     <row r="36" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>46</v>
@@ -2727,10 +2728,10 @@
         <v>1</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
@@ -2745,7 +2746,7 @@
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="N36" s="5"/>
       <c r="O36" s="5"/>
@@ -2768,16 +2769,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -2789,18 +2790,18 @@
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: remove info boxes from pdf
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC07AB00-37A2-494A-86C9-309CF3C4864A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9492D8-5148-2B46-A58A-035C1895B052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,7 +580,7 @@
  Select the level that best describes how AI was used in developing this activity.</t>
   </si>
   <si>
-    <t>affirmed: I affirm that I have critically reviewed, verified, and substantively revised any AI-assisted content in this activity. My own intellectual and creative contribution to this activity is substantial enough that I hold copyright in the final work, and I accept full responsibility for the accuracy, originality, instructional design, and POGIL alignment of the submitted activity.</t>
+    <t>affirmed: I have critically reviewed, verified, and substantively revised any AI-assisted content in this activity. My own intellectual and creative contribution to this activity is substantial enough that I hold copyright in the final work, and I accept full responsibility for the accuracy, originality, instructional design, and POGIL alignment of the submitted activity.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
break up kind, review, and posting goal
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875E7DAF-12FE-F64A-9B7C-37E42B7A870B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C9803A-D6AD-CF4C-8B89-08C8D7F15F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="189">
   <si>
     <t>PAC Activity Submission Form — Structure Specification</t>
   </si>
@@ -596,6 +596,15 @@
 • TRADITIONAL REVIEW: Reviewers provide written feedback based on the appropriate rubric.
 • COLLABORATIVE ACTIVITY FEEDBACK: Authors meet virtually and share feedback with each other in a facilitated session.
 • CLASSROOM TESTING: Activities are sent to testers, who provide feedback based on their classroom experiences.</t>
+  </si>
+  <si>
+    <t>Kind of Feedback</t>
+  </si>
+  <si>
+    <t>kind_of_feedback</t>
+  </si>
+  <si>
+    <t>posting_goal_intro</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1130,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1172,43 +1181,43 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="B4" s="5">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>35</v>
+    <row r="4" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>186</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="5">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>37</v>
+      <c r="C5" t="s">
+        <v>89</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B6" s="5">
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>32</v>
@@ -1216,58 +1225,86 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="5">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="5">
-        <v>9</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="5">
-        <v>10</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B10" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="5">
+        <v>10</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1422,7 +1459,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1562,12 +1599,12 @@
       <c r="A4" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>33</v>
+      <c r="B4" t="s">
+        <v>187</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>185</v>
@@ -1594,12 +1631,12 @@
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>33</v>
+      <c r="B5" t="s">
+        <v>187</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>85</v>
@@ -1629,26 +1666,24 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="70" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="56" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>91</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
         <v>83</v>
       </c>
@@ -1660,30 +1695,30 @@
         <v>32</v>
       </c>
       <c r="L6" s="5"/>
-      <c r="M6" s="5" t="s">
-        <v>92</v>
-      </c>
+      <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" ht="56" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>168</v>
+        <v>88</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>166</v>
+        <v>88</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="G7" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="H7" s="5" t="s">
         <v>83</v>
       </c>
@@ -1695,32 +1730,29 @@
         <v>32</v>
       </c>
       <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="56" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>93</v>
+        <v>168</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>94</v>
+        <v>181</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>95</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="G8" s="5"/>
       <c r="H8" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>83</v>
@@ -1736,23 +1768,23 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>90</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>82</v>
@@ -1769,35 +1801,33 @@
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
     </row>
-    <row r="10" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>169</v>
+        <v>97</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>90</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>173</v>
+        <v>98</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
         <v>32</v>
       </c>
@@ -1808,23 +1838,23 @@
     </row>
     <row r="11" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>90</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>83</v>
@@ -1845,23 +1875,23 @@
     </row>
     <row r="12" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>90</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>83</v>
@@ -1880,25 +1910,25 @@
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
     </row>
-    <row r="13" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>166</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>90</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>83</v>
@@ -1907,7 +1937,7 @@
         <v>83</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>103</v>
+        <v>43</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>32</v>
@@ -1917,33 +1947,35 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>58</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="C14" s="5"/>
       <c r="D14" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>105</v>
+        <v>172</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G14" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>176</v>
+      </c>
       <c r="H14" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="J14" s="5"/>
+        <v>83</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="K14" s="5" t="s">
         <v>32</v>
       </c>
@@ -1954,7 +1986,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>30</v>
@@ -1963,13 +1995,13 @@
         <v>58</v>
       </c>
       <c r="D15" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
@@ -1989,7 +2021,7 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>30</v>
@@ -1998,20 +2030,20 @@
         <v>58</v>
       </c>
       <c r="D16" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5" t="s">
@@ -2022,28 +2054,28 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
     </row>
-    <row r="17" spans="1:15" ht="70" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="D17" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>115</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="G17" s="5"/>
       <c r="H17" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>83</v>
@@ -2053,31 +2085,29 @@
         <v>32</v>
       </c>
       <c r="L17" s="5"/>
-      <c r="M17" s="5" t="s">
-        <v>165</v>
-      </c>
+      <c r="M17" s="5"/>
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="140" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ht="70" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>82</v>
@@ -2090,29 +2120,31 @@
         <v>32</v>
       </c>
       <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="M18" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ht="140" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>82</v>
@@ -2131,22 +2163,24 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G20" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>122</v>
+      </c>
       <c r="H20" s="5" t="s">
         <v>82</v>
       </c>
@@ -2162,26 +2196,24 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
     </row>
-    <row r="21" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>127</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
         <v>82</v>
       </c>
@@ -2197,24 +2229,26 @@
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>28</v>
+        <v>125</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G22" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="H22" s="5" t="s">
         <v>82</v>
       </c>
@@ -2232,20 +2266,20 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>178</v>
+        <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
@@ -2265,29 +2299,27 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>65</v>
-      </c>
+      <c r="C24" s="5"/>
       <c r="D24" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="5" t="s">
         <v>82</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5" t="s">
@@ -2300,19 +2332,19 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D25" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>106</v>
@@ -2335,116 +2367,114 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="5"/>
+        <v>36</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="D26" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="G26" s="5"/>
       <c r="H26" s="5" t="s">
         <v>82</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J26" s="5"/>
       <c r="K26" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L26" s="5"/>
-      <c r="M26" s="5" t="s">
-        <v>134</v>
-      </c>
+      <c r="M26" s="5"/>
       <c r="N26" s="5"/>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5">
         <v>1</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>177</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="J27" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="J27" s="5"/>
       <c r="K27" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
+      <c r="M27" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
     </row>
     <row r="28" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>61</v>
-      </c>
+      <c r="C28" s="5"/>
       <c r="D28" s="5">
         <v>1</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>62</v>
+        <v>136</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G28" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>177</v>
+      </c>
       <c r="H28" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="J28" s="5"/>
+      <c r="J28" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="K28" s="5" t="s">
         <v>32</v>
       </c>
       <c r="L28" s="5"/>
-      <c r="M28" s="5" t="s">
-        <v>138</v>
-      </c>
+      <c r="M28" s="5"/>
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
     </row>
     <row r="29" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>47</v>
@@ -2453,17 +2483,15 @@
         <v>61</v>
       </c>
       <c r="D29" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>140</v>
+        <v>62</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>141</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="G29" s="5"/>
       <c r="H29" s="5" t="s">
         <v>82</v>
       </c>
@@ -2475,13 +2503,15 @@
         <v>32</v>
       </c>
       <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
+      <c r="M29" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
     </row>
     <row r="30" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>47</v>
@@ -2490,17 +2520,19 @@
         <v>61</v>
       </c>
       <c r="D30" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="H30" s="5" t="s">
-        <v>144</v>
+        <v>82</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>83</v>
@@ -2509,33 +2541,33 @@
       <c r="K30" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L30" s="5" t="s">
-        <v>145</v>
-      </c>
+      <c r="L30" s="5"/>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
       <c r="O30" s="5"/>
     </row>
-    <row r="31" spans="1:15" ht="306" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C31" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="D31" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>179</v>
+        <v>143</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>147</v>
+        <v>106</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="5" t="s">
-        <v>83</v>
+        <v>144</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>83</v>
@@ -2544,33 +2576,33 @@
       <c r="K31" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L31" s="5"/>
+      <c r="L31" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
       <c r="O31" s="5"/>
     </row>
-    <row r="32" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="306" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>150</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="G32" s="5"/>
       <c r="H32" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>83</v>
@@ -2584,28 +2616,28 @@
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
     </row>
-    <row r="33" spans="1:15" ht="84" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>144</v>
+        <v>82</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>83</v>
@@ -2614,31 +2646,31 @@
       <c r="K33" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L33" s="5" t="s">
-        <v>151</v>
-      </c>
+      <c r="L33" s="5"/>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
       <c r="O33" s="5"/>
     </row>
-    <row r="34" spans="1:15" ht="28" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="84" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="G34" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>180</v>
+      </c>
       <c r="H34" s="5" t="s">
         <v>144</v>
       </c>
@@ -2656,26 +2688,26 @@
       <c r="N34" s="5"/>
       <c r="O34" s="5"/>
     </row>
-    <row r="35" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>133</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>83</v>
@@ -2684,12 +2716,47 @@
       <c r="K35" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5" t="s">
-        <v>159</v>
-      </c>
+      <c r="L35" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="M35" s="5"/>
       <c r="N35" s="5"/>
       <c r="O35" s="5"/>
+    </row>
+    <row r="36" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5">
+        <v>1</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: copyright section expanded
</commit_message>
<xml_diff>
--- a/structure.xlsx
+++ b/structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/GitHub/pac-submission-form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B168C2-DD0D-064B-B4E0-4E33DE3C97DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B80E7C-7EF5-CA44-99AE-F75265730CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="201">
   <si>
     <t>field_id</t>
   </si>
@@ -76,6 +76,13 @@
   </si>
   <si>
     <t>submission_kind</t>
+  </si>
+  <si>
+    <t>The PAC supports activity writing across all stages of development. What is your estimate for the stage of your activity?
+• ACTIVITY IDEAS are ideas, intial drafts, rough activities. Authors are seeking collaborators to work on these ideas to develop activities.
+• ACTIVITIES FOR REVIEW are complete activities. Authors are seeking formative feedback to improve the quality of the activity. 
+• ACTIVITIES FOR TESTING are complete learning cycle or application activities that are ready for widespread classroom testing. Authors are seeking classroom testing feedback to optimize the activity.  
+• APPROVED ACTIVITIES are polished activities that have been revised based on classroom testing and meet the The POGIL Project's standards for a "high-quality activity."</t>
   </si>
   <si>
     <t>info</t>
@@ -252,6 +259,12 @@
     <t>tel</t>
   </si>
   <si>
+    <t>author_institution</t>
+  </si>
+  <si>
+    <t>Institution</t>
+  </si>
+  <si>
     <t>activity_type</t>
   </si>
   <si>
@@ -372,49 +385,46 @@
     <t>500 words or less</t>
   </si>
   <si>
-    <t>image_authorship_mode</t>
-  </si>
-  <si>
-    <t>image_source</t>
-  </si>
-  <si>
-    <t>Image Authorship</t>
-  </si>
-  <si>
-    <t>blanket_author:I am the author of all images in the activity|specify:Specify image authorship individually</t>
+    <t>copyright_authorship_mode</t>
+  </si>
+  <si>
+    <t>copyright_attribution</t>
+  </si>
+  <si>
+    <t>Copyrighted Materials</t>
+  </si>
+  <si>
+    <t>blanket_author:I am the sole author of all materials in this activity|specify:Specify authorship individually</t>
   </si>
   <si>
     <t>approved_activity</t>
   </si>
   <si>
-    <t>image_description</t>
-  </si>
-  <si>
-    <t>image_source_group</t>
-  </si>
-  <si>
-    <t>Image</t>
-  </si>
-  <si>
-    <t>A short description or filename identifying the image.</t>
-  </si>
-  <si>
-    <t>image_role</t>
-  </si>
-  <si>
-    <t>Image Credit</t>
-  </si>
-  <si>
-    <t>author:I am the author of this image|source:I am not the author of this image. Image source:</t>
-  </si>
-  <si>
-    <t>image_source_detail</t>
+    <t>item_description</t>
+  </si>
+  <si>
+    <t>copyright_item_group</t>
+  </si>
+  <si>
+    <t>Brief description or filename of the copyrighted material (e.g. Figure 3 from Smith 2020, or data_table.csv)</t>
+  </si>
+  <si>
+    <t>item_role</t>
+  </si>
+  <si>
+    <t>Authorship</t>
+  </si>
+  <si>
+    <t>author:I am the author of this material|source:I am not the author of this material. Source:</t>
+  </si>
+  <si>
+    <t>item_source_detail</t>
   </si>
   <si>
     <t>Source (URL or description)</t>
   </si>
   <si>
-    <t>image_role == 'source'</t>
+    <t>item_role == 'source'</t>
   </si>
   <si>
     <t>ai_use_intro</t>
@@ -571,7 +581,7 @@
     <t>Classroom Testing &amp; Revision</t>
   </si>
   <si>
-    <t>Image Source</t>
+    <t>Copyright &amp; Attribution</t>
   </si>
   <si>
     <t>Generative AI Use</t>
@@ -598,10 +608,13 @@
     <t>+ Add another author</t>
   </si>
   <si>
-    <t>+ Add image</t>
-  </si>
-  <si>
-    <t>image_authorship_mode == 'specify'</t>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>+ Add item</t>
+  </si>
+  <si>
+    <t>copyright_authorship_mode == 'specify'</t>
   </si>
   <si>
     <t>+ Add content objective</t>
@@ -628,17 +641,12 @@
     <t>Start of editorial content: submission kind</t>
   </si>
   <si>
-    <t>The PAC supports activity writing across all stages of development. What is your estimate for the stage of your activity?
-• ACTIVITY IDEAS are ideas, intial drafts, rough activities. Authors are seeking collaborators to work on these ideas to develop activities.
-• ACTIVITIES FOR REVIEW are complete activities. Authors are seeking formative feedback to improve the quality of the activity. 
-• ACTIVITIES FOR TESTING are complete learning cycle or application activities that are ready for widespread classroom testing. Authors are seeking classroom testing feedback to optimize the activity.  
-• APPROVED ACTIVITIES are polished activities that have been revised based on classroom testing and meet the The POGIL Project's standards for a "high-quality activity."</t>
-  </si>
-  <si>
-    <t>author_institution</t>
-  </si>
-  <si>
-    <t>Institution</t>
+    <t>copyright_intro</t>
+  </si>
+  <si>
+    <t>The standards for including copyrighted materials changes as activities move toward Approval. 
+• APPROVED ACTIVITIES: the author(s) should hold copyright on all materials OR specifically identify the origin of materials that would require a license. 
+• REVIEW and TESTING: Activities may use copyrighted materials with proper attribution under Fair Use.</t>
   </si>
 </sst>
 </file>
@@ -1051,95 +1059,95 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1162,12 +1170,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1195,10 +1203,10 @@
         <v>3</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>10</v>
@@ -1206,7 +1214,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
@@ -1215,10 +1223,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1232,15 +1240,15 @@
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1249,15 +1257,15 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1266,15 +1274,15 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B6" s="5">
         <v>5</v>
@@ -1283,15 +1291,15 @@
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B7" s="5">
         <v>6</v>
@@ -1300,15 +1308,15 @@
         <v>3</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1317,15 +1325,15 @@
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -1334,15 +1342,15 @@
         <v>5</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B10" s="5">
         <v>9</v>
@@ -1351,15 +1359,15 @@
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B11" s="5">
         <v>10</v>
@@ -1368,15 +1376,15 @@
         <v>7</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -1385,10 +1393,10 @@
         <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1422,16 +1430,16 @@
         <v>3</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>9</v>
@@ -1442,96 +1450,96 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>64</v>
       </c>
       <c r="C2" s="5">
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E2" s="5">
         <v>1</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C3" s="5">
         <v>2</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>121</v>
+        <v>188</v>
       </c>
       <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E4" s="5">
         <v>1</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C5" s="5">
         <v>3</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E5" s="5">
         <v>1</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -1543,7 +1551,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1622,21 +1630,21 @@
         <v>1</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>196</v>
+        <v>17</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
@@ -1645,7 +1653,7 @@
     </row>
     <row r="3" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>16</v>
@@ -1655,57 +1663,57 @@
         <v>2</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L3" s="5"/>
       <c r="N3" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" ht="154" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5">
         <v>1</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L4" s="5"/>
       <c r="N4" s="5"/>
@@ -1713,70 +1721,70 @@
     </row>
     <row r="5" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5">
         <v>2</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5">
         <v>1</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
@@ -1785,33 +1793,33 @@
     </row>
     <row r="7" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5">
         <v>2</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L7" s="5"/>
       <c r="N7" s="5"/>
@@ -1819,31 +1827,31 @@
     </row>
     <row r="8" spans="1:15" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5">
         <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
@@ -1852,33 +1860,33 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5">
         <v>2</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
@@ -1887,33 +1895,33 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5">
         <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
@@ -1922,35 +1930,35 @@
     </row>
     <row r="11" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5">
         <v>4</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
@@ -1959,35 +1967,35 @@
     </row>
     <row r="12" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5">
         <v>5</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
@@ -1996,35 +2004,35 @@
     </row>
     <row r="13" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5">
         <v>6</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
@@ -2033,35 +2041,35 @@
     </row>
     <row r="14" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5">
         <v>7</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
@@ -2070,33 +2078,33 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" s="5">
         <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
@@ -2105,33 +2113,33 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D16" s="5">
         <v>2</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
@@ -2140,33 +2148,33 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" s="5">
         <v>3</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
@@ -2175,33 +2183,33 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>197</v>
+        <v>75</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D18" s="5">
         <v>4</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>198</v>
+        <v>76</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="J18" s="5"/>
       <c r="K18" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
@@ -2210,70 +2218,70 @@
     </row>
     <row r="19" spans="1:15" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5">
         <v>1</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
     </row>
     <row r="20" spans="1:15" ht="140" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5">
         <v>3</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
@@ -2282,62 +2290,62 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D21">
         <v>3.5</v>
       </c>
       <c r="E21" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H21" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="I21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L21" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5">
         <v>4</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
@@ -2346,66 +2354,66 @@
     </row>
     <row r="23" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5">
         <v>5</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5">
         <v>6</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
@@ -2414,31 +2422,31 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5">
         <v>1</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J25" s="5"/>
       <c r="K25" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
@@ -2447,31 +2455,31 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5">
         <v>2</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G26" s="5"/>
       <c r="H26" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J26" s="5"/>
       <c r="K26" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
@@ -2480,33 +2488,33 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D27" s="5">
         <v>3</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
@@ -2515,33 +2523,33 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D28" s="5">
         <v>4</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -2550,106 +2558,94 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5">
         <v>5</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J29" s="5"/>
       <c r="K29" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
     </row>
     <row r="30" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5">
         <v>1</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J30" s="5"/>
       <c r="K30" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L30" s="5"/>
       <c r="M30" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N30" s="5"/>
       <c r="O30" s="5"/>
     </row>
     <row r="31" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>114</v>
+        <v>199</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5">
         <v>1</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I31" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="K31" s="5" t="s">
-        <v>19</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -2657,289 +2653,326 @@
     </row>
     <row r="32" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5">
+        <v>2</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="F32" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G32" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D32" s="5">
-        <v>1</v>
-      </c>
-      <c r="E32" s="5" t="s">
+      <c r="H32" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J32" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="F32" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J32" s="5"/>
       <c r="K32" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L32" s="5"/>
-      <c r="M32" s="5" t="s">
-        <v>122</v>
-      </c>
+      <c r="M32" s="5"/>
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="D33" s="5">
+        <v>3</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D33" s="5">
-        <v>2</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="F33" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>125</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
+      <c r="M33" s="5" t="s">
+        <v>124</v>
+      </c>
       <c r="N33" s="5"/>
       <c r="O33" s="5"/>
     </row>
-    <row r="34" spans="1:15" ht="306" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D34" s="5">
         <v>3</v>
       </c>
       <c r="E34" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G34" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="F34" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J34" s="5"/>
       <c r="K34" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L34" s="5" t="s">
-        <v>128</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="L34" s="5"/>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
       <c r="O34" s="5"/>
     </row>
-    <row r="35" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="5">
+        <v>4</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5">
-        <v>1</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>131</v>
-      </c>
       <c r="F35" s="5" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L35" s="5"/>
+        <v>20</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>130</v>
+      </c>
       <c r="M35" s="5"/>
       <c r="N35" s="5"/>
       <c r="O35" s="5"/>
     </row>
-    <row r="36" spans="1:15" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>132</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>130</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="5" t="s">
         <v>133</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>134</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
       <c r="N36" s="5"/>
       <c r="O36" s="5"/>
     </row>
-    <row r="37" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" ht="84" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E37" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>137</v>
-      </c>
       <c r="H37" s="5" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J37" s="5"/>
       <c r="K37" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L37" s="5" t="s">
-        <v>138</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="L37" s="5"/>
       <c r="M37" s="5"/>
       <c r="N37" s="5"/>
       <c r="O37" s="5"/>
     </row>
-    <row r="38" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="G38" s="5"/>
+        <v>45</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>139</v>
+      </c>
       <c r="H38" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="M38" s="5"/>
       <c r="N38" s="5"/>
       <c r="O38" s="5"/>
     </row>
-    <row r="39" spans="1:15" ht="42" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>141</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L39" s="5"/>
-      <c r="M39" s="5" t="s">
-        <v>144</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="L39" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="M39" s="5"/>
       <c r="N39" s="5"/>
       <c r="O39" s="5"/>
+    </row>
+    <row r="40" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5">
+        <v>1</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L40" s="5"/>
+      <c r="M40" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="N40" s="5"/>
+      <c r="O40" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2959,40 +2992,40 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="9" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>